<commit_message>
Remove Notes column from intermediate and product import templates
</commit_message>
<xml_diff>
--- a/client/public/templates/PriceRight_Intermediates_Import_Template.xlsx
+++ b/client/public/templates/PriceRight_Intermediates_Import_Template.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A70"/>
+  <dimension ref="A1:A66"/>
   <cols>
     <col min="1" max="1" width="100.83203125" customWidth="1"/>
   </cols>
@@ -720,49 +720,29 @@
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v xml:space="preserve">  Notes — Optional</v>
+        <v>SAMPLE DATA:</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v xml:space="preserve">    Any additional notes</v>
+        <v>The Import Data sheet contains sample rows showing the correct format.</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v xml:space="preserve">    Example: Yield-based processing</v>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" t="str">
-        <v>SAMPLE DATA:</v>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" t="str">
-        <v>The Import Data sheet contains sample rows showing the correct format.</v>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" t="str">
         <v>Delete them before importing.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A70"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A66"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:I5"/>
   <cols>
     <col min="1" max="1" width="21.83203125" customWidth="1"/>
     <col min="2" max="2" width="18.83203125" customWidth="1"/>
@@ -773,7 +753,6 @@
     <col min="7" max="7" width="18.83203125" customWidth="1"/>
     <col min="8" max="8" width="18.83203125" customWidth="1"/>
     <col min="9" max="9" width="22.83203125" customWidth="1"/>
-    <col min="10" max="10" width="18.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -804,9 +783,6 @@
       <c r="I1" t="str">
         <v>Component Quantity</v>
       </c>
-      <c r="J1" t="str">
-        <v>Notes</v>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -836,9 +812,6 @@
       <c r="I2">
         <v>25</v>
       </c>
-      <c r="J2" t="str">
-        <v>First component — main ingredient</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -868,9 +841,6 @@
       <c r="I3">
         <v>0.5</v>
       </c>
-      <c r="J3" t="str">
-        <v>Second component — same intermediate</v>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -900,9 +870,6 @@
       <c r="I4">
         <v>7</v>
       </c>
-      <c r="J4" t="str">
-        <v>Third row — different intermediate</v>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -932,13 +899,10 @@
       <c r="I5">
         <v>1.5</v>
       </c>
-      <c r="J5" t="str">
-        <v>Fourth row — second component</v>
-      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I5"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>